<commit_message>
Normalize Chemprop scaffold fallback values
</commit_message>
<xml_diff>
--- a/samples/public_review_demo/discovery/ranked_hypothesis_candidates_review.xlsx
+++ b/samples/public_review_demo/discovery/ranked_hypothesis_candidates_review.xlsx
@@ -929,7 +929,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ7" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ8" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ9" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ10" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ11" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>["chemprop_v2_scaffolded_not_active", "external_imported_model_not_configured"]</t>
+          <t>["chemprop_v2_scaffold_not_active", "external_imported_model_not_configured"]</t>
         </is>
       </c>
       <c r="AJ13" t="inlineStr">
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="4">

</xml_diff>